<commit_message>
Fix 30.08 order: cluster main/доп columns, correct omelet substitution
Column layout now matches the established convention (premium main,
standard main, доп adjacent, then their exceptions) instead of
splitting the standard main away from доп with exception columns in
between. Dropped the redundant "ОСНОВНОЙ ЗАКАЗ" label on the single-
group table 9 column.

Also fixed an invented "omelet without peas" variant: the kitchen only
ever serves two omelet forms (standard/lactose-free), so that exclusion
now falls back to yogurt instead. Documented this as a standing rule in
composition.py for future orders.
</commit_message>
<xml_diff>
--- a/output/Гонконг 30.08.2026 (обработка).xlsx
+++ b/output/Гонконг 30.08.2026 (обработка).xlsx
@@ -713,44 +713,44 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
+          <t>ОСНОВНОЙ ЗАКАЗ</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>ДОП</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
           <t>БЕЗ МОЛОЧКИ, БЕЗ ГЛЮТЕНА</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>БЕЗ СВИНИНЫ</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>БЕЗ КАШ</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>БЕЗ МОЛОЧКИ, БЕЗ ЛУКА, БЕЗ ГЛЮТЕНА, БЕЗ МОРКОВКИ, БЕЗ РИСА</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>БЕЗ СЫРОЙ МОРКОВИ, ГОРОХА, ЯБЛОК</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>БЕЗ РЫБЫ</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>ОСНОВНОЙ ЗАКАЗ</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>ДОП</t>
-        </is>
-      </c>
       <c r="V2" s="3" t="inlineStr">
         <is>
           <t>БЕЗ РЫБЫ</t>
@@ -761,11 +761,7 @@
           <t>БЕЗ САХАРА, РИСА И ПЕЧЕНИ</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>ОСНОВНОЙ ЗАКАЗ</t>
-        </is>
-      </c>
+      <c r="X2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="46.5" customHeight="1">
       <c r="A3" s="6" t="n"/>
@@ -919,10 +915,10 @@
         <v>15</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>1</v>
@@ -937,10 +933,10 @@
         <v>1</v>
       </c>
       <c r="T4" s="9" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="U4" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V4" s="9" t="n">
         <v>1</v>
@@ -1105,21 +1101,21 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N6" s="15" t="n"/>
+      <c r="N6" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O6" s="15">
         <f>O4</f>
         <v/>
       </c>
       <c r="P6" s="15" t="n"/>
-      <c r="Q6" s="15" t="n"/>
-      <c r="R6" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S6" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="Q6" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R6" s="15" t="n"/>
+      <c r="S6" s="15" t="n"/>
       <c r="T6" s="15">
         <f>T4</f>
         <v/>
@@ -1162,18 +1158,18 @@
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
       <c r="M7" s="9" t="n"/>
-      <c r="N7" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N7" s="9" t="n"/>
       <c r="O7" s="9" t="n"/>
-      <c r="P7" s="9" t="n"/>
-      <c r="Q7" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P7" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q7" s="9" t="n"/>
       <c r="R7" s="9" t="n"/>
-      <c r="S7" s="9" t="n"/>
+      <c r="S7" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T7" s="9" t="n"/>
       <c r="U7" s="9" t="n"/>
       <c r="V7" s="9" t="n"/>
@@ -1264,24 +1260,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N9" s="15" t="n"/>
+      <c r="N9" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O9" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P9" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q9" s="15" t="n"/>
+      <c r="P9" s="15" t="n"/>
+      <c r="Q9" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R9" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S9" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S9" s="15" t="n"/>
       <c r="T9" s="15">
         <f>T4</f>
         <v/>
@@ -1321,18 +1317,18 @@
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
       <c r="M10" s="9" t="n"/>
-      <c r="N10" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N10" s="9" t="n"/>
       <c r="O10" s="9" t="n"/>
-      <c r="P10" s="9" t="n"/>
-      <c r="Q10" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P10" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q10" s="9" t="n"/>
       <c r="R10" s="9" t="n"/>
-      <c r="S10" s="9" t="n"/>
+      <c r="S10" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T10" s="9" t="n"/>
       <c r="U10" s="9" t="n"/>
       <c r="V10" s="9" t="n"/>
@@ -1387,25 +1383,25 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N11" s="15" t="n"/>
+      <c r="N11" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O11" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P11" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q11" s="15" t="n"/>
-      <c r="R11" s="15" t="n"/>
-      <c r="S11" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T11" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
+      <c r="P11" s="15" t="n"/>
+      <c r="Q11" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R11" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S11" s="15" t="n"/>
+      <c r="T11" s="15" t="n"/>
       <c r="U11" s="15">
         <f>U4</f>
         <v/>
@@ -1447,18 +1443,18 @@
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
       <c r="M12" s="9" t="n"/>
-      <c r="N12" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N12" s="9" t="n"/>
       <c r="O12" s="9" t="n"/>
-      <c r="P12" s="9" t="n"/>
-      <c r="Q12" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P12" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q12" s="9" t="n"/>
       <c r="R12" s="9" t="n"/>
-      <c r="S12" s="9" t="n"/>
+      <c r="S12" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T12" s="9" t="n"/>
       <c r="U12" s="9" t="n"/>
       <c r="V12" s="9" t="n"/>
@@ -1469,7 +1465,7 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>ОМЛЕТ ОВОЩНОЙ БЕЗ ГОРОШКА</t>
+          <t>ЙОГУРТ</t>
         </is>
       </c>
       <c r="C13" s="9">
@@ -1490,12 +1486,12 @@
       <c r="O13" s="9" t="n"/>
       <c r="P13" s="9" t="n"/>
       <c r="Q13" s="9" t="n"/>
-      <c r="R13" s="9">
-        <f>R4</f>
-        <v/>
-      </c>
+      <c r="R13" s="9" t="n"/>
       <c r="S13" s="9" t="n"/>
-      <c r="T13" s="9" t="n"/>
+      <c r="T13" s="9">
+        <f>T4</f>
+        <v/>
+      </c>
       <c r="U13" s="9" t="n"/>
       <c r="V13" s="9" t="n"/>
       <c r="W13" s="9" t="n"/>
@@ -1546,24 +1542,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N14" s="15" t="n"/>
+      <c r="N14" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O14" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P14" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q14" s="15" t="n"/>
+      <c r="P14" s="15" t="n"/>
+      <c r="Q14" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R14" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S14" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S14" s="15" t="n"/>
       <c r="T14" s="15">
         <f>T4</f>
         <v/>
@@ -1624,24 +1620,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N15" s="15" t="n"/>
+      <c r="N15" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O15" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P15" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q15" s="15" t="n"/>
+      <c r="P15" s="15" t="n"/>
+      <c r="Q15" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R15" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S15" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S15" s="15" t="n"/>
       <c r="T15" s="15">
         <f>T4</f>
         <v/>
@@ -2105,15 +2101,15 @@
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R20" s="15" t="n"/>
+      <c r="R20" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
       <c r="S20" s="15">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T20" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
+      <c r="T20" s="15" t="n"/>
       <c r="U20" s="15">
         <f>U4</f>
         <v/>
@@ -2156,12 +2152,12 @@
       <c r="O21" s="9" t="n"/>
       <c r="P21" s="9" t="n"/>
       <c r="Q21" s="9" t="n"/>
-      <c r="R21" s="9">
-        <f>R4</f>
-        <v/>
-      </c>
+      <c r="R21" s="9" t="n"/>
       <c r="S21" s="9" t="n"/>
-      <c r="T21" s="9" t="n"/>
+      <c r="T21" s="9">
+        <f>T4</f>
+        <v/>
+      </c>
       <c r="U21" s="9" t="n"/>
       <c r="V21" s="9" t="n"/>
       <c r="W21" s="9" t="n"/>
@@ -2653,15 +2649,15 @@
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q28" s="15" t="n"/>
+      <c r="Q28" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R28" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S28" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S28" s="15" t="n"/>
       <c r="T28" s="15">
         <f>T4</f>
         <v/>
@@ -2707,12 +2703,12 @@
       <c r="N29" s="9" t="n"/>
       <c r="O29" s="9" t="n"/>
       <c r="P29" s="9" t="n"/>
-      <c r="Q29" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="Q29" s="9" t="n"/>
       <c r="R29" s="9" t="n"/>
-      <c r="S29" s="9" t="n"/>
+      <c r="S29" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T29" s="9" t="n"/>
       <c r="U29" s="9" t="n"/>
       <c r="V29" s="9" t="n"/>
@@ -2770,24 +2766,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N30" s="15" t="n"/>
+      <c r="N30" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O30" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P30" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q30" s="15" t="n"/>
+      <c r="P30" s="15" t="n"/>
+      <c r="Q30" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R30" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S30" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S30" s="15" t="n"/>
       <c r="T30" s="15">
         <f>T4</f>
         <v/>
@@ -2830,18 +2826,18 @@
       <c r="K31" s="9" t="n"/>
       <c r="L31" s="9" t="n"/>
       <c r="M31" s="9" t="n"/>
-      <c r="N31" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N31" s="9" t="n"/>
       <c r="O31" s="9" t="n"/>
-      <c r="P31" s="9" t="n"/>
-      <c r="Q31" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P31" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q31" s="9" t="n"/>
       <c r="R31" s="9" t="n"/>
-      <c r="S31" s="9" t="n"/>
+      <c r="S31" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T31" s="9" t="n"/>
       <c r="U31" s="9" t="n"/>
       <c r="V31" s="9" t="n"/>
@@ -3112,24 +3108,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N35" s="15" t="n"/>
+      <c r="N35" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O35" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P35" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q35" s="15" t="n"/>
+      <c r="P35" s="15" t="n"/>
+      <c r="Q35" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R35" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S35" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S35" s="15" t="n"/>
       <c r="T35" s="15">
         <f>T4</f>
         <v/>
@@ -3433,24 +3429,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N39" s="15" t="n"/>
+      <c r="N39" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O39" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P39" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q39" s="15" t="n"/>
+      <c r="P39" s="15" t="n"/>
+      <c r="Q39" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R39" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S39" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S39" s="15" t="n"/>
       <c r="T39" s="15">
         <f>T4</f>
         <v/>
@@ -3490,18 +3486,18 @@
       <c r="K40" s="9" t="n"/>
       <c r="L40" s="9" t="n"/>
       <c r="M40" s="9" t="n"/>
-      <c r="N40" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N40" s="9" t="n"/>
       <c r="O40" s="9" t="n"/>
-      <c r="P40" s="9" t="n"/>
-      <c r="Q40" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P40" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q40" s="9" t="n"/>
       <c r="R40" s="9" t="n"/>
-      <c r="S40" s="9" t="n"/>
+      <c r="S40" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T40" s="9" t="n"/>
       <c r="U40" s="9" t="n"/>
       <c r="V40" s="9" t="n"/>
@@ -3844,24 +3840,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N44" s="15" t="n"/>
+      <c r="N44" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O44" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P44" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q44" s="15" t="n"/>
+      <c r="P44" s="15" t="n"/>
+      <c r="Q44" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R44" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S44" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S44" s="15" t="n"/>
       <c r="T44" s="15">
         <f>T4</f>
         <v/>
@@ -3913,18 +3909,18 @@
       <c r="K45" s="9" t="n"/>
       <c r="L45" s="9" t="n"/>
       <c r="M45" s="9" t="n"/>
-      <c r="N45" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N45" s="9" t="n"/>
       <c r="O45" s="9" t="n"/>
-      <c r="P45" s="9" t="n"/>
-      <c r="Q45" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P45" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q45" s="9" t="n"/>
       <c r="R45" s="9" t="n"/>
-      <c r="S45" s="9" t="n"/>
+      <c r="S45" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T45" s="9" t="n"/>
       <c r="U45" s="9" t="n"/>
       <c r="V45" s="9" t="n"/>
@@ -3979,24 +3975,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N46" s="15" t="n"/>
+      <c r="N46" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O46" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P46" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q46" s="15" t="n"/>
+      <c r="P46" s="15" t="n"/>
+      <c r="Q46" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R46" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S46" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S46" s="15" t="n"/>
       <c r="T46" s="15">
         <f>T4</f>
         <v/>
@@ -4042,18 +4038,18 @@
       <c r="K47" s="9" t="n"/>
       <c r="L47" s="9" t="n"/>
       <c r="M47" s="9" t="n"/>
-      <c r="N47" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N47" s="9" t="n"/>
       <c r="O47" s="9" t="n"/>
-      <c r="P47" s="9" t="n"/>
-      <c r="Q47" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P47" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q47" s="9" t="n"/>
       <c r="R47" s="9" t="n"/>
-      <c r="S47" s="9" t="n"/>
+      <c r="S47" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T47" s="9" t="n"/>
       <c r="U47" s="9" t="n"/>
       <c r="V47" s="9" t="n"/>
@@ -4378,24 +4374,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N51" s="15" t="n"/>
+      <c r="N51" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O51" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P51" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q51" s="15" t="n"/>
+      <c r="P51" s="15" t="n"/>
+      <c r="Q51" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R51" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S51" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S51" s="15" t="n"/>
       <c r="T51" s="15">
         <f>T4</f>
         <v/>
@@ -4573,24 +4569,24 @@
         <f>M4</f>
         <v/>
       </c>
-      <c r="N53" s="15" t="n"/>
+      <c r="N53" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
       <c r="O53" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P53" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q53" s="15" t="n"/>
+      <c r="P53" s="15" t="n"/>
+      <c r="Q53" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
       <c r="R53" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S53" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
+      <c r="S53" s="15" t="n"/>
       <c r="T53" s="15">
         <f>T4</f>
         <v/>
@@ -4636,18 +4632,18 @@
       <c r="K54" s="9" t="n"/>
       <c r="L54" s="9" t="n"/>
       <c r="M54" s="9" t="n"/>
-      <c r="N54" s="9">
-        <f>N4</f>
-        <v/>
-      </c>
+      <c r="N54" s="9" t="n"/>
       <c r="O54" s="9" t="n"/>
-      <c r="P54" s="9" t="n"/>
-      <c r="Q54" s="9">
-        <f>Q4</f>
-        <v/>
-      </c>
+      <c r="P54" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q54" s="9" t="n"/>
       <c r="R54" s="9" t="n"/>
-      <c r="S54" s="9" t="n"/>
+      <c r="S54" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T54" s="9" t="n"/>
       <c r="U54" s="9" t="n"/>
       <c r="V54" s="9" t="n"/>

</xml_diff>

<commit_message>
Add table-9 blanket restriction: no sugar, beets, or potato
Table 9 (columns V/W/X) turns out to have a shared physical-table
restriction beyond the per-column exceptions stated in the order text:
no sugar, beets, or potato for any of its three columns. Added "свекла"
and "картофель" as tracked composition categories, widened V/W/X's
exclusions, and rerouted every affected dish (porridge, cake, bread,
sugar packets, sweetened drinks, the beet salad, and the baked potato
garnish) to a safe alternative already used elsewhere in the day's menu.
</commit_message>
<xml_diff>
--- a/output/Гонконг 30.08.2026 (обработка).xlsx
+++ b/output/Гонконг 30.08.2026 (обработка).xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X54"/>
+  <dimension ref="A1:X55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.75" customWidth="1" min="1" max="1"/>
@@ -1124,15 +1124,9 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V6" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
+      <c r="V6" s="15" t="n"/>
       <c r="W6" s="15" t="n"/>
-      <c r="X6" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="X6" s="15" t="n"/>
     </row>
     <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="1" t="n"/>
@@ -1205,12 +1199,18 @@
       <c r="S8" s="9" t="n"/>
       <c r="T8" s="9" t="n"/>
       <c r="U8" s="9" t="n"/>
-      <c r="V8" s="9" t="n"/>
+      <c r="V8" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
       <c r="W8" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X8" s="9" t="n"/>
+      <c r="X8" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="37.5" customHeight="1">
       <c r="A9" s="13" t="n"/>
@@ -1286,15 +1286,9 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V9" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
+      <c r="V9" s="15" t="n"/>
       <c r="W9" s="15" t="n"/>
-      <c r="X9" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="X9" s="15" t="n"/>
     </row>
     <row r="10" ht="37.5" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -1331,12 +1325,18 @@
       </c>
       <c r="T10" s="9" t="n"/>
       <c r="U10" s="9" t="n"/>
-      <c r="V10" s="9" t="n"/>
+      <c r="V10" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
       <c r="W10" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X10" s="9" t="n"/>
+      <c r="X10" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="37.5" customHeight="1">
       <c r="A11" s="13" t="n"/>
@@ -1568,15 +1568,9 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V14" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
+      <c r="V14" s="15" t="n"/>
       <c r="W14" s="15" t="n"/>
-      <c r="X14" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="X14" s="15" t="n"/>
     </row>
     <row r="15" ht="37.5" customHeight="1">
       <c r="A15" s="13" t="n"/>
@@ -1826,15 +1820,9 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V17" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
+      <c r="V17" s="15" t="n"/>
       <c r="W17" s="15" t="n"/>
-      <c r="X17" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="X17" s="15" t="n"/>
     </row>
     <row r="18" ht="37.5" customHeight="1">
       <c r="A18" s="13" t="n"/>
@@ -2240,15 +2228,9 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V22" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
+      <c r="V22" s="15" t="n"/>
       <c r="W22" s="15" t="n"/>
-      <c r="X22" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="X22" s="15" t="n"/>
     </row>
     <row r="23" ht="37.5" customHeight="1">
       <c r="A23" s="1" t="n"/>
@@ -2279,12 +2261,18 @@
       <c r="S23" s="9" t="n"/>
       <c r="T23" s="9" t="n"/>
       <c r="U23" s="9" t="n"/>
-      <c r="V23" s="9" t="n"/>
+      <c r="V23" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
       <c r="W23" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X23" s="9" t="n"/>
+      <c r="X23" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="37.5" customHeight="1">
       <c r="A24" s="13" t="n"/>
@@ -2927,672 +2915,615 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V32" s="15">
+      <c r="V32" s="15" t="n"/>
+      <c r="W32" s="15" t="n"/>
+      <c r="X32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="37.5" customHeight="1">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>ГРЕЧА</t>
+        </is>
+      </c>
+      <c r="C33" s="9">
+        <f>SUM(D33:X33)</f>
+        <v/>
+      </c>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="9" t="n"/>
+      <c r="L33" s="9" t="n"/>
+      <c r="M33" s="9" t="n"/>
+      <c r="N33" s="9" t="n"/>
+      <c r="O33" s="9" t="n"/>
+      <c r="P33" s="9" t="n"/>
+      <c r="Q33" s="9" t="n"/>
+      <c r="R33" s="9" t="n"/>
+      <c r="S33" s="9" t="n"/>
+      <c r="T33" s="9" t="n"/>
+      <c r="U33" s="9" t="n"/>
+      <c r="V33" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W32" s="15">
+      <c r="W33" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X32" s="15">
+      <c r="X33" s="9">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="33" ht="37.5" customHeight="1">
-      <c r="A33" s="13" t="n"/>
-      <c r="B33" s="14" t="inlineStr">
+    <row r="34" ht="37.5" customHeight="1">
+      <c r="A34" s="13" t="n"/>
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>НАПИТОК</t>
         </is>
       </c>
-      <c r="C33" s="15">
-        <f>SUM(D33:X33)</f>
-        <v/>
-      </c>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15">
+      <c r="C34" s="15">
+        <f>SUM(D34:X34)</f>
+        <v/>
+      </c>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G33" s="15">
+      <c r="G34" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H33" s="15">
+      <c r="H34" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I33" s="15">
+      <c r="I34" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J33" s="15">
+      <c r="J34" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K33" s="15">
+      <c r="K34" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L33" s="15">
+      <c r="L34" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M33" s="15">
+      <c r="M34" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N33" s="15">
+      <c r="N34" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O33" s="15">
+      <c r="O34" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P33" s="15">
+      <c r="P34" s="15">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q33" s="15">
+      <c r="Q34" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R33" s="15">
+      <c r="R34" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S33" s="15">
+      <c r="S34" s="15">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T33" s="15">
+      <c r="T34" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U33" s="15">
+      <c r="U34" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V33" s="15">
+      <c r="V34" s="15" t="n"/>
+      <c r="W34" s="15" t="n"/>
+      <c r="X34" s="15" t="n"/>
+    </row>
+    <row r="35" ht="37.5" customHeight="1">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>НАПИТОК БЕЗ САХАРА</t>
+        </is>
+      </c>
+      <c r="C35" s="9">
+        <f>SUM(D35:X35)</f>
+        <v/>
+      </c>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="9" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="9" t="n"/>
+      <c r="O35" s="9" t="n"/>
+      <c r="P35" s="9" t="n"/>
+      <c r="Q35" s="9" t="n"/>
+      <c r="R35" s="9" t="n"/>
+      <c r="S35" s="9" t="n"/>
+      <c r="T35" s="9" t="n"/>
+      <c r="U35" s="9" t="n"/>
+      <c r="V35" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W33" s="15" t="n"/>
-      <c r="X33" s="15">
+      <c r="W35" s="9">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X35" s="9">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="34" ht="37.5" customHeight="1">
-      <c r="A34" s="1" t="n"/>
-      <c r="B34" s="16" t="inlineStr">
+    <row r="36" ht="37.5" customHeight="1">
+      <c r="A36" s="13" t="n"/>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+        </is>
+      </c>
+      <c r="C36" s="15">
+        <f>SUM(D36:X36)</f>
+        <v/>
+      </c>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G36" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H36" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I36" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J36" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L36" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M36" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N36" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O36" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P36" s="15" t="n"/>
+      <c r="Q36" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R36" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S36" s="15" t="n"/>
+      <c r="T36" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U36" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V36" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W36" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X36" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="29.25" customHeight="1">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>ПОЛДНИК</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U37" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V37" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="W37" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+      <c r="X37" s="12" t="inlineStr">
+        <is>
+          <t>9 СТОЛ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="37.5" customHeight="1">
+      <c r="A38" s="13" t="n"/>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>НАПИТОК</t>
+        </is>
+      </c>
+      <c r="C38" s="15">
+        <f>SUM(D38:X38)</f>
+        <v/>
+      </c>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G38" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H38" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I38" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L38" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M38" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N38" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O38" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P38" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q38" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R38" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S38" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T38" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U38" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V38" s="15" t="n"/>
+      <c r="W38" s="15" t="n"/>
+      <c r="X38" s="15" t="n"/>
+    </row>
+    <row r="39" ht="37.5" customHeight="1">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>НАПИТОК БЕЗ САХАРА</t>
         </is>
       </c>
-      <c r="C34" s="9">
-        <f>SUM(D34:X34)</f>
-        <v/>
-      </c>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" s="9" t="n"/>
-      <c r="J34" s="9" t="n"/>
-      <c r="K34" s="9" t="n"/>
-      <c r="L34" s="9" t="n"/>
-      <c r="M34" s="9" t="n"/>
-      <c r="N34" s="9" t="n"/>
-      <c r="O34" s="9" t="n"/>
-      <c r="P34" s="9" t="n"/>
-      <c r="Q34" s="9" t="n"/>
-      <c r="R34" s="9" t="n"/>
-      <c r="S34" s="9" t="n"/>
-      <c r="T34" s="9" t="n"/>
-      <c r="U34" s="9" t="n"/>
-      <c r="V34" s="9" t="n"/>
-      <c r="W34" s="9">
+      <c r="C39" s="9">
+        <f>SUM(D39:X39)</f>
+        <v/>
+      </c>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="9" t="n"/>
+      <c r="L39" s="9" t="n"/>
+      <c r="M39" s="9" t="n"/>
+      <c r="N39" s="9" t="n"/>
+      <c r="O39" s="9" t="n"/>
+      <c r="P39" s="9" t="n"/>
+      <c r="Q39" s="9" t="n"/>
+      <c r="R39" s="9" t="n"/>
+      <c r="S39" s="9" t="n"/>
+      <c r="T39" s="9" t="n"/>
+      <c r="U39" s="9" t="n"/>
+      <c r="V39" s="9">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W39" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X34" s="9" t="n"/>
-    </row>
-    <row r="35" ht="37.5" customHeight="1">
-      <c r="A35" s="13" t="n"/>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
-        </is>
-      </c>
-      <c r="C35" s="15">
-        <f>SUM(D35:X35)</f>
-        <v/>
-      </c>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="15">
+      <c r="X39" s="9">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="37.5" customHeight="1">
+      <c r="A40" s="13" t="n"/>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ПЕЧЕНЬЕ </t>
+        </is>
+      </c>
+      <c r="C40" s="15">
+        <f>SUM(D40:X40)</f>
+        <v/>
+      </c>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="15" t="n"/>
+      <c r="F40" s="15">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G35" s="15">
+      <c r="G40" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H35" s="15">
+      <c r="H40" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I35" s="15">
+      <c r="I40" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J35" s="15">
+      <c r="J40" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K35" s="15">
+      <c r="K40" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L35" s="15">
+      <c r="L40" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M35" s="15">
+      <c r="M40" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N35" s="15">
+      <c r="N40" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O35" s="15">
+      <c r="O40" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P35" s="15" t="n"/>
-      <c r="Q35" s="15">
+      <c r="P40" s="15" t="n"/>
+      <c r="Q40" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R35" s="15">
+      <c r="R40" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S35" s="15" t="n"/>
-      <c r="T35" s="15">
+      <c r="S40" s="15" t="n"/>
+      <c r="T40" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U35" s="15">
+      <c r="U40" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V35" s="15">
+      <c r="V40" s="15" t="n"/>
+      <c r="W40" s="15" t="n"/>
+      <c r="X40" s="15" t="n"/>
+    </row>
+    <row r="41" ht="37.5" customHeight="1">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>ЯБЛОКО ЗАПЕЧЕННОЕ</t>
+        </is>
+      </c>
+      <c r="C41" s="9">
+        <f>SUM(D41:X41)</f>
+        <v/>
+      </c>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="9" t="n"/>
+      <c r="J41" s="9" t="n"/>
+      <c r="K41" s="9" t="n"/>
+      <c r="L41" s="9" t="n"/>
+      <c r="M41" s="9" t="n"/>
+      <c r="N41" s="9" t="n"/>
+      <c r="O41" s="9" t="n"/>
+      <c r="P41" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q41" s="9" t="n"/>
+      <c r="R41" s="9" t="n"/>
+      <c r="S41" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T41" s="9" t="n"/>
+      <c r="U41" s="9" t="n"/>
+      <c r="V41" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W35" s="15">
+      <c r="W41" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X35" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="29.25" customHeight="1">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>ПОЛДНИК</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="n"/>
-      <c r="D36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U36" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V36" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="W36" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-      <c r="X36" s="12" t="inlineStr">
-        <is>
-          <t>9 СТОЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="37.5" customHeight="1">
-      <c r="A37" s="13" t="n"/>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>НАПИТОК</t>
-        </is>
-      </c>
-      <c r="C37" s="15">
-        <f>SUM(D37:X37)</f>
-        <v/>
-      </c>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G37" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H37" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I37" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J37" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K37" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L37" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M37" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N37" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O37" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P37" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q37" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R37" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S37" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T37" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U37" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V37" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W37" s="15" t="n"/>
-      <c r="X37" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="37.5" customHeight="1">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>НАПИТОК БЕЗ САХАРА</t>
-        </is>
-      </c>
-      <c r="C38" s="9">
-        <f>SUM(D38:X38)</f>
-        <v/>
-      </c>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="9" t="n"/>
-      <c r="F38" s="9" t="n"/>
-      <c r="G38" s="9" t="n"/>
-      <c r="H38" s="9" t="n"/>
-      <c r="I38" s="9" t="n"/>
-      <c r="J38" s="9" t="n"/>
-      <c r="K38" s="9" t="n"/>
-      <c r="L38" s="9" t="n"/>
-      <c r="M38" s="9" t="n"/>
-      <c r="N38" s="9" t="n"/>
-      <c r="O38" s="9" t="n"/>
-      <c r="P38" s="9" t="n"/>
-      <c r="Q38" s="9" t="n"/>
-      <c r="R38" s="9" t="n"/>
-      <c r="S38" s="9" t="n"/>
-      <c r="T38" s="9" t="n"/>
-      <c r="U38" s="9" t="n"/>
-      <c r="V38" s="9" t="n"/>
-      <c r="W38" s="9">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X38" s="9" t="n"/>
-    </row>
-    <row r="39" ht="37.5" customHeight="1">
-      <c r="A39" s="13" t="n"/>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ПЕЧЕНЬЕ </t>
-        </is>
-      </c>
-      <c r="C39" s="15">
-        <f>SUM(D39:X39)</f>
-        <v/>
-      </c>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G39" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H39" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I39" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J39" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K39" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L39" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M39" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N39" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O39" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P39" s="15" t="n"/>
-      <c r="Q39" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R39" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S39" s="15" t="n"/>
-      <c r="T39" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U39" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V39" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W39" s="15" t="n"/>
-      <c r="X39" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="37.5" customHeight="1">
-      <c r="A40" s="1" t="n"/>
-      <c r="B40" s="16" t="inlineStr">
-        <is>
-          <t>ЯБЛОКО ЗАПЕЧЕННОЕ</t>
-        </is>
-      </c>
-      <c r="C40" s="9">
-        <f>SUM(D40:X40)</f>
-        <v/>
-      </c>
-      <c r="D40" s="9" t="n"/>
-      <c r="E40" s="9" t="n"/>
-      <c r="F40" s="9" t="n"/>
-      <c r="G40" s="9" t="n"/>
-      <c r="H40" s="9" t="n"/>
-      <c r="I40" s="9" t="n"/>
-      <c r="J40" s="9" t="n"/>
-      <c r="K40" s="9" t="n"/>
-      <c r="L40" s="9" t="n"/>
-      <c r="M40" s="9" t="n"/>
-      <c r="N40" s="9" t="n"/>
-      <c r="O40" s="9" t="n"/>
-      <c r="P40" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q40" s="9" t="n"/>
-      <c r="R40" s="9" t="n"/>
-      <c r="S40" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T40" s="9" t="n"/>
-      <c r="U40" s="9" t="n"/>
-      <c r="V40" s="9" t="n"/>
-      <c r="W40" s="9">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X40" s="9" t="n"/>
-    </row>
-    <row r="41" ht="37.5" customHeight="1">
-      <c r="A41" s="13" t="n"/>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>ЧАЙ</t>
-        </is>
-      </c>
-      <c r="C41" s="15">
-        <f>SUM(D41:X41)</f>
-        <v/>
-      </c>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G41" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H41" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I41" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J41" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K41" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L41" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M41" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N41" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O41" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P41" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q41" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R41" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S41" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T41" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U41" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V41" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W41" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X41" s="15">
+      <c r="X41" s="9">
         <f>X4</f>
         <v/>
       </c>
@@ -3601,7 +3532,7 @@
       <c r="A42" s="13" t="n"/>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
+          <t>ЧАЙ</t>
         </is>
       </c>
       <c r="C42" s="15">
@@ -3678,493 +3609,487 @@
         <f>V4</f>
         <v/>
       </c>
-      <c r="W42" s="15" t="n"/>
+      <c r="W42" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
       <c r="X42" s="15">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="43" ht="29.25" customHeight="1">
-      <c r="A43" s="10" t="n"/>
-      <c r="B43" s="11" t="inlineStr">
+    <row r="43" ht="37.5" customHeight="1">
+      <c r="A43" s="13" t="n"/>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>САХАР ПОРЦИОННЫЙ</t>
+        </is>
+      </c>
+      <c r="C43" s="15">
+        <f>SUM(D43:X43)</f>
+        <v/>
+      </c>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G43" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H43" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I43" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J43" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K43" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L43" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M43" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N43" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O43" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P43" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q43" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R43" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S43" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T43" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U43" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V43" s="15" t="n"/>
+      <c r="W43" s="15" t="n"/>
+      <c r="X43" s="15" t="n"/>
+    </row>
+    <row r="44" ht="29.25" customHeight="1">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>УЖИН</t>
         </is>
       </c>
-      <c r="C43" s="10" t="n"/>
-      <c r="D43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U43" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V43" s="12" t="inlineStr">
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U44" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V44" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
-      <c r="W43" s="12" t="inlineStr">
+      <c r="W44" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
-      <c r="X43" s="12" t="inlineStr">
+      <c r="X44" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="37.5" customHeight="1">
-      <c r="A44" s="13" t="n"/>
-      <c r="B44" s="14" t="inlineStr">
+    <row r="45" ht="37.5" customHeight="1">
+      <c r="A45" s="13" t="n"/>
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>САЛАТ СВЕКОЛЬНЫЙ С СЫРНЫМ МУССОМ</t>
         </is>
       </c>
-      <c r="C44" s="15">
-        <f>SUM(D44:X44)</f>
-        <v/>
-      </c>
-      <c r="D44" s="15">
+      <c r="C45" s="15">
+        <f>SUM(D45:X45)</f>
+        <v/>
+      </c>
+      <c r="D45" s="15">
         <f>D4</f>
         <v/>
       </c>
-      <c r="E44" s="15">
+      <c r="E45" s="15">
         <f>E4</f>
         <v/>
       </c>
-      <c r="F44" s="15" t="n"/>
-      <c r="G44" s="15">
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H44" s="15" t="n"/>
-      <c r="I44" s="15" t="n"/>
-      <c r="J44" s="15">
+      <c r="H45" s="15" t="n"/>
+      <c r="I45" s="15" t="n"/>
+      <c r="J45" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K44" s="15">
+      <c r="K45" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L44" s="15">
+      <c r="L45" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M44" s="15">
+      <c r="M45" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N44" s="15">
+      <c r="N45" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O44" s="15">
+      <c r="O45" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P44" s="15" t="n"/>
-      <c r="Q44" s="15">
+      <c r="P45" s="15" t="n"/>
+      <c r="Q45" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R44" s="15">
+      <c r="R45" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S44" s="15" t="n"/>
-      <c r="T44" s="15">
+      <c r="S45" s="15" t="n"/>
+      <c r="T45" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U44" s="15">
+      <c r="U45" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V44" s="15">
+      <c r="V45" s="15" t="n"/>
+      <c r="W45" s="15" t="n"/>
+      <c r="X45" s="15" t="n"/>
+    </row>
+    <row r="46" ht="37.5" customHeight="1">
+      <c r="A46" s="1" t="n"/>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>ОВОЩНОЙ САЛАТ</t>
+        </is>
+      </c>
+      <c r="C46" s="9">
+        <f>SUM(D46:X46)</f>
+        <v/>
+      </c>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I46" s="9">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J46" s="9" t="n"/>
+      <c r="K46" s="9" t="n"/>
+      <c r="L46" s="9" t="n"/>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="9" t="n"/>
+      <c r="O46" s="9" t="n"/>
+      <c r="P46" s="9">
+        <f>P4</f>
+        <v/>
+      </c>
+      <c r="Q46" s="9" t="n"/>
+      <c r="R46" s="9" t="n"/>
+      <c r="S46" s="9">
+        <f>S4</f>
+        <v/>
+      </c>
+      <c r="T46" s="9" t="n"/>
+      <c r="U46" s="9" t="n"/>
+      <c r="V46" s="9">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W44" s="15">
+      <c r="W46" s="9">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X44" s="15">
+      <c r="X46" s="9">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="45" ht="37.5" customHeight="1">
-      <c r="A45" s="1" t="n"/>
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>ОВОЩНОЙ САЛАТ</t>
-        </is>
-      </c>
-      <c r="C45" s="9">
-        <f>SUM(D45:X45)</f>
-        <v/>
-      </c>
-      <c r="D45" s="9" t="n"/>
-      <c r="E45" s="9" t="n"/>
-      <c r="F45" s="9">
+    <row r="47" ht="37.5" customHeight="1">
+      <c r="A47" s="13" t="n"/>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>РУЛЕТ КУРИНЫЙ С СЫРОМ И БРОККОЛИ</t>
+        </is>
+      </c>
+      <c r="C47" s="15">
+        <f>SUM(D47:X47)</f>
+        <v/>
+      </c>
+      <c r="D47" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E47" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H47" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I47" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J47" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K47" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L47" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M47" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N47" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O47" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P47" s="15" t="n"/>
+      <c r="Q47" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R47" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S47" s="15" t="n"/>
+      <c r="T47" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U47" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V47" s="15">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="W47" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="X47" s="15">
+        <f>X4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="37.5" customHeight="1">
+      <c r="A48" s="1" t="n"/>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>ИНДЕЙКА ГРУДКА</t>
+        </is>
+      </c>
+      <c r="C48" s="9">
+        <f>SUM(D48:X48)</f>
+        <v/>
+      </c>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="9">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G45" s="9" t="n"/>
-      <c r="H45" s="9">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I45" s="9">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J45" s="9" t="n"/>
-      <c r="K45" s="9" t="n"/>
-      <c r="L45" s="9" t="n"/>
-      <c r="M45" s="9" t="n"/>
-      <c r="N45" s="9" t="n"/>
-      <c r="O45" s="9" t="n"/>
-      <c r="P45" s="9">
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="9" t="n"/>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="9" t="n"/>
+      <c r="O48" s="9" t="n"/>
+      <c r="P48" s="9">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q45" s="9" t="n"/>
-      <c r="R45" s="9" t="n"/>
-      <c r="S45" s="9">
+      <c r="Q48" s="9" t="n"/>
+      <c r="R48" s="9" t="n"/>
+      <c r="S48" s="9">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T45" s="9" t="n"/>
-      <c r="U45" s="9" t="n"/>
-      <c r="V45" s="9" t="n"/>
-      <c r="W45" s="9" t="n"/>
-      <c r="X45" s="9" t="n"/>
-    </row>
-    <row r="46" ht="37.5" customHeight="1">
-      <c r="A46" s="13" t="n"/>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>РУЛЕТ КУРИНЫЙ С СЫРОМ И БРОККОЛИ</t>
-        </is>
-      </c>
-      <c r="C46" s="15">
-        <f>SUM(D46:X46)</f>
-        <v/>
-      </c>
-      <c r="D46" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E46" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F46" s="15" t="n"/>
-      <c r="G46" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H46" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I46" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J46" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K46" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L46" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M46" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N46" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O46" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P46" s="15" t="n"/>
-      <c r="Q46" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R46" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S46" s="15" t="n"/>
-      <c r="T46" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U46" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V46" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W46" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X46" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="37.5" customHeight="1">
-      <c r="A47" s="1" t="n"/>
-      <c r="B47" s="16" t="inlineStr">
-        <is>
-          <t>ИНДЕЙКА ГРУДКА</t>
-        </is>
-      </c>
-      <c r="C47" s="9">
-        <f>SUM(D47:X47)</f>
-        <v/>
-      </c>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
-      <c r="F47" s="9">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G47" s="9" t="n"/>
-      <c r="H47" s="9" t="n"/>
-      <c r="I47" s="9" t="n"/>
-      <c r="J47" s="9" t="n"/>
-      <c r="K47" s="9" t="n"/>
-      <c r="L47" s="9" t="n"/>
-      <c r="M47" s="9" t="n"/>
-      <c r="N47" s="9" t="n"/>
-      <c r="O47" s="9" t="n"/>
-      <c r="P47" s="9">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q47" s="9" t="n"/>
-      <c r="R47" s="9" t="n"/>
-      <c r="S47" s="9">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T47" s="9" t="n"/>
-      <c r="U47" s="9" t="n"/>
-      <c r="V47" s="9" t="n"/>
-      <c r="W47" s="9" t="n"/>
-      <c r="X47" s="9" t="n"/>
-    </row>
-    <row r="48" ht="37.5" customHeight="1">
-      <c r="A48" s="13" t="n"/>
-      <c r="B48" s="14" t="inlineStr">
-        <is>
-          <t>ГРЕЧА</t>
-        </is>
-      </c>
-      <c r="C48" s="15">
-        <f>SUM(D48:X48)</f>
-        <v/>
-      </c>
-      <c r="D48" s="15">
-        <f>D4</f>
-        <v/>
-      </c>
-      <c r="E48" s="15">
-        <f>E4</f>
-        <v/>
-      </c>
-      <c r="F48" s="15">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="G48" s="15">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="H48" s="15">
-        <f>H4</f>
-        <v/>
-      </c>
-      <c r="I48" s="15">
-        <f>I4</f>
-        <v/>
-      </c>
-      <c r="J48" s="15">
-        <f>J4</f>
-        <v/>
-      </c>
-      <c r="K48" s="15">
-        <f>K4</f>
-        <v/>
-      </c>
-      <c r="L48" s="15">
-        <f>L4</f>
-        <v/>
-      </c>
-      <c r="M48" s="15">
-        <f>M4</f>
-        <v/>
-      </c>
-      <c r="N48" s="15">
-        <f>N4</f>
-        <v/>
-      </c>
-      <c r="O48" s="15">
-        <f>O4</f>
-        <v/>
-      </c>
-      <c r="P48" s="15">
-        <f>P4</f>
-        <v/>
-      </c>
-      <c r="Q48" s="15">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="R48" s="15">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="S48" s="15">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="T48" s="15">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="U48" s="15">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="V48" s="15">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="W48" s="15">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="X48" s="15">
-        <f>X4</f>
-        <v/>
-      </c>
+      <c r="T48" s="9" t="n"/>
+      <c r="U48" s="9" t="n"/>
+      <c r="V48" s="9" t="n"/>
+      <c r="W48" s="9" t="n"/>
+      <c r="X48" s="9" t="n"/>
     </row>
     <row r="49" ht="37.5" customHeight="1">
       <c r="A49" s="13" t="n"/>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>ЧАЙ</t>
+          <t>ГРЕЧА</t>
         </is>
       </c>
       <c r="C49" s="15">
         <f>SUM(D49:X49)</f>
         <v/>
       </c>
-      <c r="D49" s="15" t="n"/>
-      <c r="E49" s="15" t="n"/>
+      <c r="D49" s="15">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="E49" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F49" s="15">
         <f>F4</f>
         <v/>
@@ -4246,7 +4171,7 @@
       <c r="A50" s="13" t="n"/>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>САХАР ПОРЦИОННЫЙ</t>
+          <t>ЧАЙ</t>
         </is>
       </c>
       <c r="C50" s="15">
@@ -4323,7 +4248,10 @@
         <f>V4</f>
         <v/>
       </c>
-      <c r="W50" s="15" t="n"/>
+      <c r="W50" s="15">
+        <f>W4</f>
+        <v/>
+      </c>
       <c r="X50" s="15">
         <f>X4</f>
         <v/>
@@ -4333,7 +4261,7 @@
       <c r="A51" s="13" t="n"/>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+          <t>САХАР ПОРЦИОННЫЙ</t>
         </is>
       </c>
       <c r="C51" s="15">
@@ -4382,7 +4310,10 @@
         <f>O4</f>
         <v/>
       </c>
-      <c r="P51" s="15" t="n"/>
+      <c r="P51" s="15">
+        <f>P4</f>
+        <v/>
+      </c>
       <c r="Q51" s="15">
         <f>Q4</f>
         <v/>
@@ -4391,7 +4322,10 @@
         <f>R4</f>
         <v/>
       </c>
-      <c r="S51" s="15" t="n"/>
+      <c r="S51" s="15">
+        <f>S4</f>
+        <v/>
+      </c>
       <c r="T51" s="15">
         <f>T4</f>
         <v/>
@@ -4400,255 +4334,330 @@
         <f>U4</f>
         <v/>
       </c>
-      <c r="V51" s="15">
+      <c r="V51" s="15" t="n"/>
+      <c r="W51" s="15" t="n"/>
+      <c r="X51" s="15" t="n"/>
+    </row>
+    <row r="52" ht="37.5" customHeight="1">
+      <c r="A52" s="13" t="n"/>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ХЛЕБ РЖАНО-ПШЕНИЧНЫЙ </t>
+        </is>
+      </c>
+      <c r="C52" s="15">
+        <f>SUM(D52:X52)</f>
+        <v/>
+      </c>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="G52" s="15">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="H52" s="15">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="I52" s="15">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="J52" s="15">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="K52" s="15">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="L52" s="15">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M52" s="15">
+        <f>M4</f>
+        <v/>
+      </c>
+      <c r="N52" s="15">
+        <f>N4</f>
+        <v/>
+      </c>
+      <c r="O52" s="15">
+        <f>O4</f>
+        <v/>
+      </c>
+      <c r="P52" s="15" t="n"/>
+      <c r="Q52" s="15">
+        <f>Q4</f>
+        <v/>
+      </c>
+      <c r="R52" s="15">
+        <f>R4</f>
+        <v/>
+      </c>
+      <c r="S52" s="15" t="n"/>
+      <c r="T52" s="15">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="U52" s="15">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="V52" s="15">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W51" s="15">
+      <c r="W52" s="15">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X51" s="15">
+      <c r="X52" s="15">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="52" ht="29.25" customHeight="1">
-      <c r="A52" s="10" t="n"/>
-      <c r="B52" s="11" t="inlineStr">
+    <row r="53" ht="29.25" customHeight="1">
+      <c r="A53" s="10" t="n"/>
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>2-Й УЖИН</t>
         </is>
       </c>
-      <c r="C52" s="10" t="n"/>
-      <c r="D52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="F52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="G52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="H52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="I52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="J52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="K52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="L52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="M52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="N52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="O52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="P52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="Q52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="R52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="S52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="T52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="U52" s="12" t="inlineStr">
-        <is>
-          <t>15 СТОЛ</t>
-        </is>
-      </c>
-      <c r="V52" s="12" t="inlineStr">
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="L53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="M53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="N53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="O53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="P53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="Q53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="R53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="S53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="T53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="U53" s="12" t="inlineStr">
+        <is>
+          <t>15 СТОЛ</t>
+        </is>
+      </c>
+      <c r="V53" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
-      <c r="W52" s="12" t="inlineStr">
+      <c r="W53" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
-      <c r="X52" s="12" t="inlineStr">
+      <c r="X53" s="12" t="inlineStr">
         <is>
           <t>9 СТОЛ</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="37.5" customHeight="1">
-      <c r="A53" s="13" t="n"/>
-      <c r="B53" s="14" t="inlineStr">
+    <row r="54" ht="37.5" customHeight="1">
+      <c r="A54" s="13" t="n"/>
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>КЕФИР</t>
         </is>
       </c>
-      <c r="C53" s="15">
-        <f>SUM(D53:X53)</f>
-        <v/>
-      </c>
-      <c r="D53" s="15" t="n"/>
-      <c r="E53" s="15" t="n"/>
-      <c r="F53" s="15" t="n"/>
-      <c r="G53" s="15">
+      <c r="C54" s="15">
+        <f>SUM(D54:X54)</f>
+        <v/>
+      </c>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="15" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="15">
         <f>G4</f>
         <v/>
       </c>
-      <c r="H53" s="15">
+      <c r="H54" s="15">
         <f>H4</f>
         <v/>
       </c>
-      <c r="I53" s="15">
+      <c r="I54" s="15">
         <f>I4</f>
         <v/>
       </c>
-      <c r="J53" s="15">
+      <c r="J54" s="15">
         <f>J4</f>
         <v/>
       </c>
-      <c r="K53" s="15">
+      <c r="K54" s="15">
         <f>K4</f>
         <v/>
       </c>
-      <c r="L53" s="15">
+      <c r="L54" s="15">
         <f>L4</f>
         <v/>
       </c>
-      <c r="M53" s="15">
+      <c r="M54" s="15">
         <f>M4</f>
         <v/>
       </c>
-      <c r="N53" s="15">
+      <c r="N54" s="15">
         <f>N4</f>
         <v/>
       </c>
-      <c r="O53" s="15">
+      <c r="O54" s="15">
         <f>O4</f>
         <v/>
       </c>
-      <c r="P53" s="15" t="n"/>
-      <c r="Q53" s="15">
+      <c r="P54" s="15" t="n"/>
+      <c r="Q54" s="15">
         <f>Q4</f>
         <v/>
       </c>
-      <c r="R53" s="15">
+      <c r="R54" s="15">
         <f>R4</f>
         <v/>
       </c>
-      <c r="S53" s="15" t="n"/>
-      <c r="T53" s="15">
+      <c r="S54" s="15" t="n"/>
+      <c r="T54" s="15">
         <f>T4</f>
         <v/>
       </c>
-      <c r="U53" s="15">
+      <c r="U54" s="15">
         <f>U4</f>
         <v/>
       </c>
-      <c r="V53" s="15">
+      <c r="V54" s="15">
         <f>V4</f>
         <v/>
       </c>
-      <c r="W53" s="15">
+      <c r="W54" s="15">
         <f>W4</f>
         <v/>
       </c>
-      <c r="X53" s="15">
+      <c r="X54" s="15">
         <f>X4</f>
         <v/>
       </c>
     </row>
-    <row r="54" ht="37.5" customHeight="1">
-      <c r="A54" s="1" t="n"/>
-      <c r="B54" s="16" t="inlineStr">
+    <row r="55" ht="37.5" customHeight="1">
+      <c r="A55" s="1" t="n"/>
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>НАПИТОК</t>
         </is>
       </c>
-      <c r="C54" s="9">
-        <f>SUM(D54:X54)</f>
-        <v/>
-      </c>
-      <c r="D54" s="9" t="n"/>
-      <c r="E54" s="9" t="n"/>
-      <c r="F54" s="9">
+      <c r="C55" s="9">
+        <f>SUM(D55:X55)</f>
+        <v/>
+      </c>
+      <c r="D55" s="9" t="n"/>
+      <c r="E55" s="9" t="n"/>
+      <c r="F55" s="9">
         <f>F4</f>
         <v/>
       </c>
-      <c r="G54" s="9" t="n"/>
-      <c r="H54" s="9" t="n"/>
-      <c r="I54" s="9" t="n"/>
-      <c r="J54" s="9" t="n"/>
-      <c r="K54" s="9" t="n"/>
-      <c r="L54" s="9" t="n"/>
-      <c r="M54" s="9" t="n"/>
-      <c r="N54" s="9" t="n"/>
-      <c r="O54" s="9" t="n"/>
-      <c r="P54" s="9">
+      <c r="G55" s="9" t="n"/>
+      <c r="H55" s="9" t="n"/>
+      <c r="I55" s="9" t="n"/>
+      <c r="J55" s="9" t="n"/>
+      <c r="K55" s="9" t="n"/>
+      <c r="L55" s="9" t="n"/>
+      <c r="M55" s="9" t="n"/>
+      <c r="N55" s="9" t="n"/>
+      <c r="O55" s="9" t="n"/>
+      <c r="P55" s="9">
         <f>P4</f>
         <v/>
       </c>
-      <c r="Q54" s="9" t="n"/>
-      <c r="R54" s="9" t="n"/>
-      <c r="S54" s="9">
+      <c r="Q55" s="9" t="n"/>
+      <c r="R55" s="9" t="n"/>
+      <c r="S55" s="9">
         <f>S4</f>
         <v/>
       </c>
-      <c r="T54" s="9" t="n"/>
-      <c r="U54" s="9" t="n"/>
-      <c r="V54" s="9" t="n"/>
-      <c r="W54" s="9" t="n"/>
-      <c r="X54" s="9" t="n"/>
+      <c r="T55" s="9" t="n"/>
+      <c r="U55" s="9" t="n"/>
+      <c r="V55" s="9" t="n"/>
+      <c r="W55" s="9" t="n"/>
+      <c r="X55" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix same-day lunch/dinner dish duplicates for 30.08 exception columns
ОВОЩНОЙ САЛАТ was reused as both the lunch salad (everyone) and the
dinner salad alternative for the beet-restricted columns - the same
client would get an identical salad twice in one day. Same issue for
ГРЕЧА, reused as both the dinner garnish (everyone) and the lunch
garnish alternative for table 9. Swapped in genuinely different dishes
already present in the recipe data (САЛАТ ЗЕЛЕНЫЙ С КУКУРУЗОЙ, СПАГЕТТИ)
so no course repeats within the same day for any column.
</commit_message>
<xml_diff>
--- a/output/Гонконг 30.08.2026 (обработка).xlsx
+++ b/output/Гонконг 30.08.2026 (обработка).xlsx
@@ -2923,7 +2923,7 @@
       <c r="A33" s="1" t="n"/>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>ГРЕЧА</t>
+          <t>СПАГЕТТИ</t>
         </is>
       </c>
       <c r="C33" s="9">
@@ -3889,7 +3889,7 @@
       <c r="A46" s="1" t="n"/>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>ОВОЩНОЙ САЛАТ</t>
+          <t>САЛАТ ЗЕЛЕНЫЙ С КУКУРУЗОЙ</t>
         </is>
       </c>
       <c r="C46" s="9">

</xml_diff>